<commit_message>
Study progress: seen counts, batch errors and Known flags
Amir's own drilling, not a code change - kept as its own commit so the
history says which is which.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/PTE_Vocabulary_Master.xlsx
+++ b/data/PTE_Vocabulary_Master.xlsx
@@ -996,10 +996,10 @@
         <v>Happening by lucky chance</v>
       </c>
       <c r="D35" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>play</v>
       </c>
     </row>
     <row r="36">
@@ -3478,10 +3478,10 @@
         <v>Cannot be replaced</v>
       </c>
       <c r="D181" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="E181" t="str">
-        <v/>
+        <v>play</v>
       </c>
     </row>
     <row r="182">
@@ -5266,70 +5266,72 @@
     <hyperlink ref="E22" r:id="rId10" tooltip="Play &quot;Deficient&quot; on Google Translate"/>
     <hyperlink ref="E25" r:id="rId11" tooltip="Play &quot;Dissuade&quot; on Google Translate"/>
     <hyperlink ref="E28" r:id="rId12" tooltip="Play &quot;Ephemeral&quot; on Google Translate"/>
-    <hyperlink ref="E37" r:id="rId13" tooltip="Play &quot;Germane&quot; on Google Translate"/>
-    <hyperlink ref="E43" r:id="rId14" tooltip="Play &quot;Hypothetical&quot; on Google Translate"/>
-    <hyperlink ref="E47" r:id="rId15" tooltip="Play &quot;Impediment&quot; on Google Translate"/>
-    <hyperlink ref="E49" r:id="rId16" tooltip="Play &quot;Implicit&quot; on Google Translate"/>
-    <hyperlink ref="E51" r:id="rId17" tooltip="Play &quot;Inapt&quot; on Google Translate"/>
-    <hyperlink ref="E52" r:id="rId18" tooltip="Play &quot;Incisive&quot; on Google Translate"/>
-    <hyperlink ref="E53" r:id="rId19" tooltip="Play &quot;Incongruous&quot; on Google Translate"/>
-    <hyperlink ref="E54" r:id="rId20" tooltip="Play &quot;Incumbent&quot; on Google Translate"/>
-    <hyperlink ref="E55" r:id="rId21" tooltip="Play &quot;Indifferent&quot; on Google Translate"/>
-    <hyperlink ref="E67" r:id="rId22" tooltip="Play &quot;Inhibit&quot; on Google Translate"/>
-    <hyperlink ref="E69" r:id="rId23" tooltip="Play &quot;Injudicious&quot; on Google Translate"/>
-    <hyperlink ref="E71" r:id="rId24" tooltip="Play &quot;Innovation&quot; on Google Translate"/>
-    <hyperlink ref="E75" r:id="rId25" tooltip="Play &quot;Insult&quot; on Google Translate"/>
-    <hyperlink ref="E86" r:id="rId26" tooltip="Play &quot;Intelligible&quot; on Google Translate"/>
-    <hyperlink ref="E91" r:id="rId27" tooltip="Play &quot;Interaction&quot; on Google Translate"/>
-    <hyperlink ref="E95" r:id="rId28" tooltip="Play &quot;Interim&quot; on Google Translate"/>
-    <hyperlink ref="E96" r:id="rId29" tooltip="Play &quot;Interior&quot; on Google Translate"/>
-    <hyperlink ref="E97" r:id="rId30" tooltip="Play &quot;Interlude&quot; on Google Translate"/>
-    <hyperlink ref="E98" r:id="rId31" tooltip="Play &quot;Interminable&quot; on Google Translate"/>
-    <hyperlink ref="E103" r:id="rId32" tooltip="Play &quot;Interpose&quot; on Google Translate"/>
-    <hyperlink ref="E105" r:id="rId33" tooltip="Play &quot;Interrogate&quot; on Google Translate"/>
-    <hyperlink ref="E108" r:id="rId34" tooltip="Play &quot;Intertwine&quot; on Google Translate"/>
-    <hyperlink ref="E109" r:id="rId35" tooltip="Play &quot;Interval&quot; on Google Translate"/>
-    <hyperlink ref="E118" r:id="rId36" tooltip="Play &quot;Intricate&quot; on Google Translate"/>
-    <hyperlink ref="E124" r:id="rId37" tooltip="Play &quot;Intrude&quot; on Google Translate"/>
-    <hyperlink ref="E125" r:id="rId38" tooltip="Play &quot;Intrusion&quot; on Google Translate"/>
-    <hyperlink ref="E127" r:id="rId39" tooltip="Play &quot;Intuitive&quot; on Google Translate"/>
-    <hyperlink ref="E130" r:id="rId40" tooltip="Play &quot;Invade&quot; on Google Translate"/>
-    <hyperlink ref="E136" r:id="rId41" tooltip="Play &quot;Invective&quot; on Google Translate"/>
-    <hyperlink ref="E139" r:id="rId42" tooltip="Play &quot;Invent&quot; on Google Translate"/>
-    <hyperlink ref="E147" r:id="rId43" tooltip="Play &quot;Investigate&quot; on Google Translate"/>
-    <hyperlink ref="E149" r:id="rId44" tooltip="Play &quot;Investiture&quot; on Google Translate"/>
-    <hyperlink ref="E151" r:id="rId45" tooltip="Play &quot;Inveterate&quot; on Google Translate"/>
-    <hyperlink ref="E154" r:id="rId46" tooltip="Play &quot;Invincible&quot; on Google Translate"/>
-    <hyperlink ref="E158" r:id="rId47" tooltip="Play &quot;Invite&quot; on Google Translate"/>
-    <hyperlink ref="E159" r:id="rId48" tooltip="Play &quot;Inviting&quot; on Google Translate"/>
-    <hyperlink ref="E160" r:id="rId49" tooltip="Play &quot;Invocation&quot; on Google Translate"/>
-    <hyperlink ref="E165" r:id="rId50" tooltip="Play &quot;Involved&quot; on Google Translate"/>
-    <hyperlink ref="E166" r:id="rId51" tooltip="Play &quot;Invulnerable&quot; on Google Translate"/>
-    <hyperlink ref="E169" r:id="rId52" tooltip="Play &quot;Irascible&quot; on Google Translate"/>
-    <hyperlink ref="E170" r:id="rId53" tooltip="Play &quot;Iridescent&quot; on Google Translate"/>
-    <hyperlink ref="E179" r:id="rId54" tooltip="Play &quot;Irreligious&quot; on Google Translate"/>
-    <hyperlink ref="E180" r:id="rId55" tooltip="Play &quot;Irreparable&quot; on Google Translate"/>
-    <hyperlink ref="E182" r:id="rId56" tooltip="Play &quot;Irrepressible&quot; on Google Translate"/>
-    <hyperlink ref="E194" r:id="rId57" tooltip="Play &quot;Irritant&quot; on Google Translate"/>
-    <hyperlink ref="E198" r:id="rId58" tooltip="Play &quot;Isolated&quot; on Google Translate"/>
-    <hyperlink ref="E222" r:id="rId59" tooltip="Play &quot;Jangle&quot; on Google Translate"/>
-    <hyperlink ref="E226" r:id="rId60" tooltip="Play &quot;Jargon&quot; on Google Translate"/>
-    <hyperlink ref="E228" r:id="rId61" tooltip="Play &quot;Jaundiced&quot; on Google Translate"/>
-    <hyperlink ref="E243" r:id="rId62" tooltip="Play &quot;Jeering&quot; on Google Translate"/>
-    <hyperlink ref="E244" r:id="rId63" tooltip="Play &quot;Jejune&quot; on Google Translate"/>
-    <hyperlink ref="E245" r:id="rId64" tooltip="Play &quot;Jell&quot; on Google Translate"/>
-    <hyperlink ref="E248" r:id="rId65" tooltip="Play &quot;Jeopardize&quot; on Google Translate"/>
-    <hyperlink ref="E249" r:id="rId66" tooltip="Play &quot;Jeopardy&quot; on Google Translate"/>
-    <hyperlink ref="E253" r:id="rId67" tooltip="Play &quot;Jerky&quot; on Google Translate"/>
-    <hyperlink ref="E258" r:id="rId68" tooltip="Play &quot;Jesus&quot; on Google Translate"/>
-    <hyperlink ref="E260" r:id="rId69" tooltip="Play &quot;Jet-black&quot; on Google Translate"/>
-    <hyperlink ref="E263" r:id="rId70" tooltip="Play &quot;Jew&quot; on Google Translate"/>
-    <hyperlink ref="E274" r:id="rId71" tooltip="Play &quot;Leisure&quot; on Google Translate"/>
-    <hyperlink ref="E275" r:id="rId72" tooltip="Play &quot;Pervades&quot; on Google Translate"/>
-    <hyperlink ref="E277" r:id="rId73" tooltip="Play &quot;Ascertain&quot; on Google Translate"/>
-    <hyperlink ref="E280" r:id="rId74" tooltip="Play &quot;Spur&quot; on Google Translate"/>
-    <hyperlink ref="E282" r:id="rId75" tooltip="Play &quot;Perspective&quot; on Google Translate"/>
-    <hyperlink ref="E283" r:id="rId76" tooltip="Play &quot;Plagiarism&quot; on Google Translate"/>
+    <hyperlink ref="E35" r:id="rId13" tooltip="Play &quot;Fortuitous&quot; on Google Translate"/>
+    <hyperlink ref="E37" r:id="rId14" tooltip="Play &quot;Germane&quot; on Google Translate"/>
+    <hyperlink ref="E43" r:id="rId15" tooltip="Play &quot;Hypothetical&quot; on Google Translate"/>
+    <hyperlink ref="E47" r:id="rId16" tooltip="Play &quot;Impediment&quot; on Google Translate"/>
+    <hyperlink ref="E49" r:id="rId17" tooltip="Play &quot;Implicit&quot; on Google Translate"/>
+    <hyperlink ref="E51" r:id="rId18" tooltip="Play &quot;Inapt&quot; on Google Translate"/>
+    <hyperlink ref="E52" r:id="rId19" tooltip="Play &quot;Incisive&quot; on Google Translate"/>
+    <hyperlink ref="E53" r:id="rId20" tooltip="Play &quot;Incongruous&quot; on Google Translate"/>
+    <hyperlink ref="E54" r:id="rId21" tooltip="Play &quot;Incumbent&quot; on Google Translate"/>
+    <hyperlink ref="E55" r:id="rId22" tooltip="Play &quot;Indifferent&quot; on Google Translate"/>
+    <hyperlink ref="E67" r:id="rId23" tooltip="Play &quot;Inhibit&quot; on Google Translate"/>
+    <hyperlink ref="E69" r:id="rId24" tooltip="Play &quot;Injudicious&quot; on Google Translate"/>
+    <hyperlink ref="E71" r:id="rId25" tooltip="Play &quot;Innovation&quot; on Google Translate"/>
+    <hyperlink ref="E75" r:id="rId26" tooltip="Play &quot;Insult&quot; on Google Translate"/>
+    <hyperlink ref="E86" r:id="rId27" tooltip="Play &quot;Intelligible&quot; on Google Translate"/>
+    <hyperlink ref="E91" r:id="rId28" tooltip="Play &quot;Interaction&quot; on Google Translate"/>
+    <hyperlink ref="E95" r:id="rId29" tooltip="Play &quot;Interim&quot; on Google Translate"/>
+    <hyperlink ref="E96" r:id="rId30" tooltip="Play &quot;Interior&quot; on Google Translate"/>
+    <hyperlink ref="E97" r:id="rId31" tooltip="Play &quot;Interlude&quot; on Google Translate"/>
+    <hyperlink ref="E98" r:id="rId32" tooltip="Play &quot;Interminable&quot; on Google Translate"/>
+    <hyperlink ref="E103" r:id="rId33" tooltip="Play &quot;Interpose&quot; on Google Translate"/>
+    <hyperlink ref="E105" r:id="rId34" tooltip="Play &quot;Interrogate&quot; on Google Translate"/>
+    <hyperlink ref="E108" r:id="rId35" tooltip="Play &quot;Intertwine&quot; on Google Translate"/>
+    <hyperlink ref="E109" r:id="rId36" tooltip="Play &quot;Interval&quot; on Google Translate"/>
+    <hyperlink ref="E118" r:id="rId37" tooltip="Play &quot;Intricate&quot; on Google Translate"/>
+    <hyperlink ref="E124" r:id="rId38" tooltip="Play &quot;Intrude&quot; on Google Translate"/>
+    <hyperlink ref="E125" r:id="rId39" tooltip="Play &quot;Intrusion&quot; on Google Translate"/>
+    <hyperlink ref="E127" r:id="rId40" tooltip="Play &quot;Intuitive&quot; on Google Translate"/>
+    <hyperlink ref="E130" r:id="rId41" tooltip="Play &quot;Invade&quot; on Google Translate"/>
+    <hyperlink ref="E136" r:id="rId42" tooltip="Play &quot;Invective&quot; on Google Translate"/>
+    <hyperlink ref="E139" r:id="rId43" tooltip="Play &quot;Invent&quot; on Google Translate"/>
+    <hyperlink ref="E147" r:id="rId44" tooltip="Play &quot;Investigate&quot; on Google Translate"/>
+    <hyperlink ref="E149" r:id="rId45" tooltip="Play &quot;Investiture&quot; on Google Translate"/>
+    <hyperlink ref="E151" r:id="rId46" tooltip="Play &quot;Inveterate&quot; on Google Translate"/>
+    <hyperlink ref="E154" r:id="rId47" tooltip="Play &quot;Invincible&quot; on Google Translate"/>
+    <hyperlink ref="E158" r:id="rId48" tooltip="Play &quot;Invite&quot; on Google Translate"/>
+    <hyperlink ref="E159" r:id="rId49" tooltip="Play &quot;Inviting&quot; on Google Translate"/>
+    <hyperlink ref="E160" r:id="rId50" tooltip="Play &quot;Invocation&quot; on Google Translate"/>
+    <hyperlink ref="E165" r:id="rId51" tooltip="Play &quot;Involved&quot; on Google Translate"/>
+    <hyperlink ref="E166" r:id="rId52" tooltip="Play &quot;Invulnerable&quot; on Google Translate"/>
+    <hyperlink ref="E169" r:id="rId53" tooltip="Play &quot;Irascible&quot; on Google Translate"/>
+    <hyperlink ref="E170" r:id="rId54" tooltip="Play &quot;Iridescent&quot; on Google Translate"/>
+    <hyperlink ref="E179" r:id="rId55" tooltip="Play &quot;Irreligious&quot; on Google Translate"/>
+    <hyperlink ref="E180" r:id="rId56" tooltip="Play &quot;Irreparable&quot; on Google Translate"/>
+    <hyperlink ref="E181" r:id="rId57" tooltip="Play &quot;Irreplaceable&quot; on Google Translate"/>
+    <hyperlink ref="E182" r:id="rId58" tooltip="Play &quot;Irrepressible&quot; on Google Translate"/>
+    <hyperlink ref="E194" r:id="rId59" tooltip="Play &quot;Irritant&quot; on Google Translate"/>
+    <hyperlink ref="E198" r:id="rId60" tooltip="Play &quot;Isolated&quot; on Google Translate"/>
+    <hyperlink ref="E222" r:id="rId61" tooltip="Play &quot;Jangle&quot; on Google Translate"/>
+    <hyperlink ref="E226" r:id="rId62" tooltip="Play &quot;Jargon&quot; on Google Translate"/>
+    <hyperlink ref="E228" r:id="rId63" tooltip="Play &quot;Jaundiced&quot; on Google Translate"/>
+    <hyperlink ref="E243" r:id="rId64" tooltip="Play &quot;Jeering&quot; on Google Translate"/>
+    <hyperlink ref="E244" r:id="rId65" tooltip="Play &quot;Jejune&quot; on Google Translate"/>
+    <hyperlink ref="E245" r:id="rId66" tooltip="Play &quot;Jell&quot; on Google Translate"/>
+    <hyperlink ref="E248" r:id="rId67" tooltip="Play &quot;Jeopardize&quot; on Google Translate"/>
+    <hyperlink ref="E249" r:id="rId68" tooltip="Play &quot;Jeopardy&quot; on Google Translate"/>
+    <hyperlink ref="E253" r:id="rId69" tooltip="Play &quot;Jerky&quot; on Google Translate"/>
+    <hyperlink ref="E258" r:id="rId70" tooltip="Play &quot;Jesus&quot; on Google Translate"/>
+    <hyperlink ref="E260" r:id="rId71" tooltip="Play &quot;Jet-black&quot; on Google Translate"/>
+    <hyperlink ref="E263" r:id="rId72" tooltip="Play &quot;Jew&quot; on Google Translate"/>
+    <hyperlink ref="E274" r:id="rId73" tooltip="Play &quot;Leisure&quot; on Google Translate"/>
+    <hyperlink ref="E275" r:id="rId74" tooltip="Play &quot;Pervades&quot; on Google Translate"/>
+    <hyperlink ref="E277" r:id="rId75" tooltip="Play &quot;Ascertain&quot; on Google Translate"/>
+    <hyperlink ref="E280" r:id="rId76" tooltip="Play &quot;Spur&quot; on Google Translate"/>
+    <hyperlink ref="E282" r:id="rId77" tooltip="Play &quot;Perspective&quot; on Google Translate"/>
+    <hyperlink ref="E283" r:id="rId78" tooltip="Play &quot;Plagiarism&quot; on Google Translate"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E285"/>

</xml_diff>